<commit_message>
fgislk: волна 16-20.09, 25 объяв (safe-append, BBL)
</commit_message>
<xml_diff>
--- a/fgislk.xlsx
+++ b/fgislk.xlsx
@@ -4648,7 +4648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE29"/>
+  <dimension ref="A1:AE32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="26"/>
@@ -8443,6 +8443,396 @@
       <c r="AE29" t="inlineStr">
         <is>
           <t>2026-10-10T14:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>5518421273</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n05/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_14_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_14_3.jpg</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Предложение услуг</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>350</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Документы на пиломатериал, ФГИС ЛК</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Занимаемся документами на пиломатериал: доска, брус, брусок, горбыль, тарная дощечка.&lt;br&gt;&lt;br&gt;После переработки учёт никуда не девается. На машину с доской нужен такой же сопроводительный документ, как на кругляк, и покупатели с бухгалтерией это спрашивают в первую очередь.&lt;br&gt;&lt;br&gt;Берём на себя: внесение объёмов в систему, оформление происхождения через договор, ЭСД с QR кодом на отгрузки, отчёт за период, закрытие расхождений по остаткам.&lt;br&gt;&lt;br&gt;Работаем с пилорамами, ИП и ООО, полностью удалённо, по всей стране.&lt;br&gt;&lt;br&gt;Напишите, что отгружаете и какой объём в месяц, посчитаем.</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Новгородская обл., Любытино, ул. Советов, 29</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Деловые услуги</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Консультирование</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>4–7 лет</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Удалённо</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Физические лица | ИП | ООО | АО | НКО | Другие юридические лица</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>2026-10-18T04:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>2026-09-18T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>2026-10-18T04:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>7039160996</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/batch/08/08_01.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_10_1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_09_1.jpg</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Предложение услуг</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>350</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Лес есть, а документов нет. Оформим</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Древесина лежит, а по бумагам её не существует. Приводим такой объём в законный вид.&lt;br&gt;&lt;br&gt;Типичные случаи: лес спилили на своём поле или на расчистке, купили у населения без оформления, объём есть в наличии, но в государственной системе учёта его нет. Продать и вывезти в таком виде нельзя.&lt;br&gt;&lt;br&gt;Что делаем: оформляем происхождение объёма через договор купли-продажи со своей стороны, заносим партию в ФГИС ЛК, ставим её вам на баланс. Дальше по каждой машине идёт сопроводительный документ с QR кодом, а за период сдаётся отчётность.&lt;br&gt;&lt;br&gt;Разбираем ситуацию бесплатно. Напишите породу, объём и откуда лес, скажем сразу, что можно сделать.</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Республика Коми, Троицко-Печорск, ул. Ленина, 2</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Деловые услуги</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Консультирование</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>4–7 лет</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Удалённо</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Физические лица | ИП | ООО | АО | НКО | Другие юридические лица</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>2026-10-19T06:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>2026-09-19T09:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>2026-10-19T06:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>4570672141</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260806/4382774059/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/batch/02/02_02.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/batch/02/02_03.jpg</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Предложение услуг</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>350</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Документы на лес и пиломатериал</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Занимаемся документами на древесину: и на круглый лес, и на пиломатериал после распиловки.&lt;br&gt;&lt;br&gt;Что обычно нужно решить. Объёма нет в системе, а продать надо. Машину не выпускают без сопроводительного документа. Подходит срок отчётности, а она не собрана. Остатки в базе разошлись с фактом, и отгрузки встали.&lt;br&gt;&lt;br&gt;По каждому пункту работаем сами: оформляем происхождение через договор купли-продажи, вносим объёмы в ФГИС ЛК, выдаём ЭСД с QR кодом, сдаём отчёт за период, закрываем расхождения.&lt;br&gt;&lt;br&gt;Работаем по всей стране удалённо, с ИП, ООО и частниками. Разбор ситуации бесплатный.</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Смоленская обл., Рославль, ул. Советская, 66</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Деловые услуги</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Консультирование</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>4–7 лет</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Удалённо</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Физические лица | ИП | ООО | АО | НКО | Другие юридические лица</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>2026-10-19T10:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>2026-09-19T13:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>2026-10-19T10:00:00+03:00</t>
         </is>
       </c>
     </row>
@@ -9095,7 +9485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK119"/>
+  <dimension ref="A1:AK139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28.33" customWidth="1" min="1" max="1"/>
@@ -25420,6 +25810,2706 @@
       <c r="AK119" t="inlineStr">
         <is>
           <t>2026-10-04T03:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>6392718516</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Берёза дрова и баланс(QR код на рейс)</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Оформляем документы на берёзу, которая уже заготовлена: дрова, баланс, кругляк с зарастающего поля.&lt;br&gt;&lt;br&gt;На каждую машину с древесиной нужен электронный сопроводительный документ с QR кодом. Без него рейс начинать рискованно, на посту это первый вопрос.&lt;br&gt;&lt;br&gt;Порядок простой. Вы пишете породу, объём, номер машины и маршрут. Мы проводим происхождение партии через договор купли-продажи, заносим объём в ФГИС ЛК и отдаём готовый документ на рейс. Обычно уходит пятнадцать минут.&lt;br&gt;&lt;br&gt;Работаем удалённо, свой кабинет в системе и электронную подпись заводить не придётся. Кто возит постоянно, берём на сопровождение помесячно.&lt;br&gt;&lt;br&gt;Берёза кругляк, дрова, баланс на комбинат, Кировская область.</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n01/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_03_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_03_3.jpg</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Кировская обл., Котельнич, ул. Ленина, 26</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P120" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W120" t="inlineStr">
+        <is>
+          <t>Берёза</t>
+        </is>
+      </c>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB120" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC120" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE120" t="inlineStr">
+        <is>
+          <t>2026-10-16T02:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF120" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH120" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI120" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ120" t="inlineStr">
+        <is>
+          <t>2026-09-16T05:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK120" t="inlineStr">
+        <is>
+          <t>2026-10-16T02:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>3073730612</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Доска обрезная, документы и ЭСД</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Документы на пиломатериал. Доска обрезная, необрезная, брусок, горбыль.&lt;br&gt;&lt;br&gt;Многие думают, что учёт касается только круглого леса. На доску сопроводительный документ нужен ровно так же, и вопросы на дороге к машине с пиломатериалом возникают не реже.&lt;br&gt;&lt;br&gt;Что делаем: заводим объём в ФГИС ЛК, оформляем происхождение через договор, готовим ЭСД с QR кодом на каждую отгрузку. Если у покупателя бухгалтерия требует полный пакет, собираем и его.&lt;br&gt;&lt;br&gt;От вас нужны порода, объём в кубах, откуда и куда едет машина. Остальное на нас, приезжать никуда не надо.&lt;br&gt;&lt;br&gt;Доска обрезная сосна и ель, пиломатериал, кругляк, Кировская область.</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n03/1.png|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_04_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_04_3.jpg</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Кировская обл., Омутнинск, ул. Комсомольская, 9</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P121" t="n">
+        <v>350</v>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>Сосна</t>
+        </is>
+      </c>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB121" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC121" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE121" t="inlineStr">
+        <is>
+          <t>2026-10-16T04:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF121" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH121" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI121" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ121" t="inlineStr">
+        <is>
+          <t>2026-09-16T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK121" t="inlineStr">
+        <is>
+          <t>2026-10-16T04:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>7628940116</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Осина баланс, QR код на вывоз</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Ставим на учёт осиновый баланс и делаем документы на вывозку.&lt;br&gt;&lt;br&gt;Осину берут плитные комбинаты, но без бумаг на происхождение партию на приёмке развернут. Отдельная история, когда лес пилили на своей земле или на расчистке, в системе такого объёма нет вообще.&lt;br&gt;&lt;br&gt;Мы это закрываем: заводим объём, оформляем договор купли-продажи как основание, дальше на каждый рейс выдаём ЭСД с QR кодом. Отчёт за период тоже готовим, если он с вас спросят.&lt;br&gt;&lt;br&gt;Объём любой, от одной машины до постоянного потока. Пишите, что и куда везёте, посчитаем сроки.&lt;br&gt;&lt;br&gt;Осина баланс, дрова, кругляк, ольха и берёза, Кировская область.</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n02/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_09_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_09_3.jpg</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Кировская обл., Яранск, ул. Кирова, 10</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P122" t="n">
+        <v>250</v>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V122" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>Осина</t>
+        </is>
+      </c>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB122" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC122" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE122" t="inlineStr">
+        <is>
+          <t>2026-10-16T06:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF122" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH122" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI122" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ122" t="inlineStr">
+        <is>
+          <t>2026-09-16T09:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK122" t="inlineStr">
+        <is>
+          <t>2026-10-16T06:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>7023394603</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Берёза баланс, ЭСД на перевозку</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Оформляем документы на берёзовый баланс и кругляк, который уже лежит на площадке.&lt;br&gt;&lt;br&gt;Без электронного сопроводительного документа машину с лесом дальше поста не пустят, а если объёма нет в системе учёта, то и сам документ выписать не из чего. Мы закрываем обе части сразу.&lt;br&gt;&lt;br&gt;Сначала проводим происхождение партии через договор купли-продажи и ставим объём вам на баланс в ФГИС ЛК. Дальше на каждый рейс выдаём ЭСД с QR кодом, обычно в течение пятнадцати минут после ваших данных.&lt;br&gt;&lt;br&gt;Подойдёт и хозяйству, которое расчищает поля, и тем, кто скупает лес у населения.&lt;br&gt;&lt;br&gt;Берёза баланс, дрова, кругляк, осина, Псковская область.</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260806/6654494961/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_20_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_20_3.jpg</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Псковская обл., Великие Луки, пр-т Ленина, 14</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P123" t="n">
+        <v>280</v>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V123" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W123" t="inlineStr">
+        <is>
+          <t>Берёза</t>
+        </is>
+      </c>
+      <c r="X123" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB123" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC123" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE123" t="inlineStr">
+        <is>
+          <t>2026-10-16T10:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF123" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH123" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI123" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ123" t="inlineStr">
+        <is>
+          <t>2026-09-16T13:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK123" t="inlineStr">
+        <is>
+          <t>2026-10-16T10:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>3195490619</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Лиственница кругляк, ЭСД на отгрузку</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Документы на лиственницу под отгрузку: машинами, вагонами, партиями на экспортёра.&lt;br&gt;&lt;br&gt;Когда объём идёт на станцию, покупатель смотрит не только на качество, но и на то, сходятся ли данные в системе. Если партия не проведена, отгрузка встаёт, и это дороже любых документов.&lt;br&gt;&lt;br&gt;Берём на себя всю цепочку: происхождение объёма через договор, внесение в ФГИС ЛК, ЭСД с QR на каждый рейс, сверка остатков перед отгрузкой. Работаем с ИП, ООО и с частниками.&lt;br&gt;&lt;br&gt;Напишите объём и куда идёт лес, разберём вашу ситуацию и скажем, что нужно.&lt;br&gt;&lt;br&gt;Лиственница кругляк, пиловочник, сосна, ель, Иркутская область.</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260806/9218798416/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_10_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_10_3.jpg</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Иркутская обл., Усть-Кут, ул. Кирова, 18</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P124" t="n">
+        <v>350</v>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V124" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>Лиственница</t>
+        </is>
+      </c>
+      <c r="X124" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB124" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC124" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE124" t="inlineStr">
+        <is>
+          <t>2026-10-17T02:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF124" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH124" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI124" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ124" t="inlineStr">
+        <is>
+          <t>2026-09-17T05:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK124" t="inlineStr">
+        <is>
+          <t>2026-10-17T02:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>8122502691</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Сосна пиловочник, документы ФГИС ЛК</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Ситуация обычная: пиловочник лежит на площадке, а в системе его нет. Мы делаем так, чтобы он там появился законно.&lt;br&gt;&lt;br&gt;Оформляем происхождение объёма договором купли-продажи, заводим партию в ФГИС ЛК, ставим её вам на баланс. После этого лес можно спокойно продавать и везти, а на каждую машину выписывать сопроводительный документ с QR кодом.&lt;br&gt;&lt;br&gt;Делаем и то, что обычно откладывают: лесную декларацию, отчёт 1-ИЛ, закрытие расхождений по остаткам.&lt;br&gt;&lt;br&gt;Всё удалённо, по всей стране. От вас порода, объём и что уже есть на руках.&lt;br&gt;&lt;br&gt;Сосна пиловочник, кругляк, баланс, ель и лиственница, Иркутская область.</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n08/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_08_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_08_3.jpg</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Иркутская обл., Усть-Илимск, ул. Героев Труда, 38</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P125" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>Сосна</t>
+        </is>
+      </c>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB125" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC125" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE125" t="inlineStr">
+        <is>
+          <t>2026-10-17T04:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF125" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH125" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI125" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ125" t="inlineStr">
+        <is>
+          <t>2026-09-17T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK125" t="inlineStr">
+        <is>
+          <t>2026-10-17T04:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>3268226363</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Ель баланс, документы на перевозку</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Возите еловый баланс на комбинат, а документы каждый раз собираются в последний момент. Забираем эту часть себе.&lt;br&gt;&lt;br&gt;Оформляем электронный сопроводительный документ на рейс, тот самый с QR кодом. Заводим объём в систему учёта древесины, если его там ещё нет, и приводим в порядок остатки, чтобы приёмка не спорила с цифрами.&lt;br&gt;&lt;br&gt;Работаем и разово, и на потоке. Для постоянных отгрузок удобнее сопровождение: вы пишете машину и объём, документ приходит в ответ, без переписки на полдня.&lt;br&gt;&lt;br&gt;Ель баланс, сосна, берёза, кругляк и дрова, Вологодская область.</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n09/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_07_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_07_3.jpg</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Вологодская обл., Великий Устюг, Советский пр-т, 100</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P126" t="n">
+        <v>280</v>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W126" t="inlineStr">
+        <is>
+          <t>Ель</t>
+        </is>
+      </c>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB126" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC126" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE126" t="inlineStr">
+        <is>
+          <t>2026-10-17T06:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF126" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH126" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI126" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ126" t="inlineStr">
+        <is>
+          <t>2026-09-17T09:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK126" t="inlineStr">
+        <is>
+          <t>2026-10-17T06:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2790722386</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Пиломатериал хвоя, QR на машину</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Делаем QR код на машину с пиломатериалом. Доска, брус, брусок, тарная дощечка.&lt;br&gt;&lt;br&gt;Вопрос, который задают чаще всего: нужен ли документ на доску, если это уже не круглый лес. Нужен. Переработка не снимает учёт, и на посту это проверяют так же.&lt;br&gt;&lt;br&gt;Оформляем быстро. Вы даёте объём, породу и маршрут, мы вносим данные и отдаём готовый ЭСД. Если объём не заведён в системе, сначала проводим происхождение через договор, это тоже наша работа.&lt;br&gt;&lt;br&gt;Пилорамам, которые отгружают регулярно, считаем помесячно, так выходит дешевле.&lt;br&gt;&lt;br&gt;Пиломатериал хвоя, доска обрезная, брус, кругляк, Вологодская область.</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260806/8757513433/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_14_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_14_3.jpg</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Вологодская обл., Тотьма, ул. Ленина, 44</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P127" t="n">
+        <v>350</v>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>Сосна</t>
+        </is>
+      </c>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB127" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC127" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE127" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF127" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH127" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI127" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ127" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK127" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>4857472831</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Сосна кругляк, QR код на вывоз</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Делаем QR код на вывоз соснового кругляка. Это тот самый электронный документ, который сейчас спрашивают на каждую машину с древесиной.&lt;br&gt;&lt;br&gt;Чаще всего к нам приходят, когда лес уже свален, покупатель найден, а бумаг на происхождение нет вообще. Оформляем их с нуля: договор купли-продажи как основание, внесение объёма в ФГИС ЛК, сопроводительный документ на рейс.&lt;br&gt;&lt;br&gt;Если остатки в системе не сходятся с фактом, приводим в порядок и это, иначе отгрузки начнут блокировать.&lt;br&gt;&lt;br&gt;Работаем удалённо, свой кабинет и электронную подпись заводить не нужно.&lt;br&gt;&lt;br&gt;Сосна кругляк, пиловочник, ель, баланс, Псковская область.</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n16/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_13_1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_13_2.jpg</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Псковская обл., Себеж, ул. 7 Ноября, 2</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P128" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W128" t="inlineStr">
+        <is>
+          <t>Сосна</t>
+        </is>
+      </c>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB128" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC128" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE128" t="inlineStr">
+        <is>
+          <t>2026-10-17T10:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF128" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH128" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI128" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ128" t="inlineStr">
+        <is>
+          <t>2026-09-17T13:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK128" t="inlineStr">
+        <is>
+          <t>2026-10-17T10:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>1762058548</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Сосна кругляк с поля, оформим учёт</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Лес, выросший на пашне или в лесополосе, по документам такой же, как из делянки. Оформляем его с нуля.&lt;br&gt;&lt;br&gt;Собственники земли часто узнают об этом уже после того, как спилили: покупатель просит бумаги, а бумаг нет, и продать несколько сотен кубов не получается.&lt;br&gt;&lt;br&gt;Мы проводим объём через договор купли-продажи, заносим в ФГИС ЛК, ставим на баланс и дальше выдаём сопроводительные документы на вывоз. В сложных случаях помогаем разобраться с назначением участка и с тем, как это правильно показать.&lt;br&gt;&lt;br&gt;Работаем удалённо, приезжать не нужно. Напишите породу и примерный объём.&lt;br&gt;&lt;br&gt;Сосна кругляк, берёза, ель, лес с сельхозземель, Новгородская область.</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n11/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_10_1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_09_1.jpg</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Новгородская обл., Чудово, ул. Некрасова, 24</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P129" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>Сосна</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB129" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE129" t="inlineStr">
+        <is>
+          <t>2026-10-18T02:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF129" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH129" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI129" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ129" t="inlineStr">
+        <is>
+          <t>2026-09-18T05:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK129" t="inlineStr">
+        <is>
+          <t>2026-10-18T02:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>4787974535</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Берёза фанкряж, ЭСД и учёт объёма</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Фанкряж и берёзовый баланс отгружают быстро, а документы тормозят всю работу. Закрываем этот кусок.&lt;br&gt;&lt;br&gt;Ставим объём на учёт в ФГИС ЛК, оформляем основание через договор купли-продажи, готовим ЭСД с QR кодом на каждую машину. Если остатки в системе разошлись с фактом, приводим их в соответствие, чтобы отгрузки не блокировались.&lt;br&gt;&lt;br&gt;Подходит и тем, у кого своя делянка, и тем, кто берёт лес у населения и не понимает, как провести такую покупку.&lt;br&gt;&lt;br&gt;От вас порода, объём, маршрут. Ответим по срокам и цене сразу.&lt;br&gt;&lt;br&gt;Берёза фанкряж, баланс, кругляк, осина, Республика Коми.</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260806/2153018262/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_03_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_03_3.jpg</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Республика Коми, Усть-Кулом, ул. Советская, 37</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P130" t="n">
+        <v>320</v>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V130" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W130" t="inlineStr">
+        <is>
+          <t>Берёза</t>
+        </is>
+      </c>
+      <c r="X130" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB130" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC130" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE130" t="inlineStr">
+        <is>
+          <t>2026-10-18T06:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF130" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH130" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI130" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ130" t="inlineStr">
+        <is>
+          <t>2026-09-18T09:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK130" t="inlineStr">
+        <is>
+          <t>2026-10-18T06:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2289536143</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Сосна кругляк, QR код за 15 минут</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Машина готова, водитель ждёт, а документа на рейс нет. Делаем его за пятнадцать минут.&lt;br&gt;&lt;br&gt;Электронный сопроводительный документ с QR кодом оформляем на любую породу и любой объём, хоть на одну машину дров, хоть на регулярные отгрузки пиловочника. Документ настоящий, виден в системе, на весовой и на посту вопросов не вызывает.&lt;br&gt;&lt;br&gt;Если объёма в системе нет, заводим его: договор купли-продажи как основание, партия на балансе, дальше рейсы.&lt;br&gt;&lt;br&gt;Нужны только данные машины, порода, объём и маршрут. Пишите в любое время, отвечаем быстро.&lt;br&gt;&lt;br&gt;Сосна кругляк, пиловочник, ель, берёза, Республика Карелия.</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260806/7393214976/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_04_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_04_3.jpg</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Республика Карелия, Пудож, ул. Ленина, 90</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P131" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V131" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W131" t="inlineStr">
+        <is>
+          <t>Сосна</t>
+        </is>
+      </c>
+      <c r="X131" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB131" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC131" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE131" t="inlineStr">
+        <is>
+          <t>2026-10-18T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF131" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH131" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI131" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ131" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK131" t="inlineStr">
+        <is>
+          <t>2026-10-18T08:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>9258836919</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Ель пиловочник, документы ФГИС ЛК</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Ставим еловый пиловочник на учёт и готовим документы под продажу.&lt;br&gt;&lt;br&gt;Покупатели с производством почти всегда просят подтверждение происхождения. Если объём не проведён в государственной системе, сделка либо срывается, либо идёт в серую, а это уже риск для обеих сторон.&lt;br&gt;&lt;br&gt;Берём весь оформительский круг на себя: договор купли-продажи, внесение партии в ФГИС ЛК, сопроводительные документы с QR кодом на каждую машину, отчётность за период.&lt;br&gt;&lt;br&gt;Пишите породу, объём и откуда лес, скажем по срокам и цене сразу.&lt;br&gt;&lt;br&gt;Ель пиловочник, сосна, кругляк, баланс, Смоленская область.</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_12_1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_11_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_13_3.jpg</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Смоленская обл., Вязьма, ул. Ленина, 14</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P132" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V132" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W132" t="inlineStr">
+        <is>
+          <t>Ель</t>
+        </is>
+      </c>
+      <c r="X132" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB132" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC132" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE132" t="inlineStr">
+        <is>
+          <t>2026-10-18T10:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF132" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH132" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI132" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ132" t="inlineStr">
+        <is>
+          <t>2026-09-18T13:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK132" t="inlineStr">
+        <is>
+          <t>2026-10-18T10:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>8693589310</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Ель пиловочник, документы на вывоз</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Разбираемся с учётом ели и готовим документы на вывоз.&lt;br&gt;&lt;br&gt;Чаще всего приходят с двумя вещами. Первая: лес заготовлен, а в системе его нет, продать официально нельзя. Вторая: объёмы когда-то внесли неверно, остатки не сходятся, и отгрузка встала.&lt;br&gt;&lt;br&gt;Закрываем и то и другое. Оформляем происхождение через договор, вносим партию в ФГИС ЛК, правим расхождения по остаткам, дальше выписываем сопроводительные документы на каждую машину.&lt;br&gt;&lt;br&gt;Работаем по всей стране удалённо, нужен только ваш объём и понимание, откуда он взялся.&lt;br&gt;&lt;br&gt;Ель пиловочник, баланс, сосна, кругляк, Костромская область.</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260806/5312403632/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_09_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_09_3.jpg</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Костромская обл., Мантурово, ул. Советская, 25</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P133" t="n">
+        <v>280</v>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V133" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W133" t="inlineStr">
+        <is>
+          <t>Ель</t>
+        </is>
+      </c>
+      <c r="X133" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB133" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC133" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE133" t="inlineStr">
+        <is>
+          <t>2026-10-19T02:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF133" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH133" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI133" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ133" t="inlineStr">
+        <is>
+          <t>2026-09-19T05:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK133" t="inlineStr">
+        <is>
+          <t>2026-10-19T02:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2543470744</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Дрова колотые, документы на продажу</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Дрова тоже древесина, и учёт для них такой же, как для делового леса. Оформляем документы тем, кто продаёт дрова машинами.&lt;br&gt;&lt;br&gt;Частника с одной машиной для себя это не касается, а вот когда возишь на продажу регулярно, нужен сопроводительный документ на рейс. Особенно если покупатель юрлицо и ему нужно провести покупку по бухгалтерии.&lt;br&gt;&lt;br&gt;Делаем полный круг: происхождение объёма, внесение в ФГИС ЛК, ЭСД с QR на каждую отгрузку, отчётность за период.&lt;br&gt;&lt;br&gt;Напишите, сколько машин в месяц возите, подберём вариант по цене.&lt;br&gt;&lt;br&gt;Дрова колотые берёза и осина, баланс, горбыль, Нижегородская область.</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/batch/05/05_01.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_10_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_10_3.jpg</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Нижегородская обл., Ветлуга, ул. Ленина, 6</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P134" t="n">
+        <v>250</v>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V134" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W134" t="inlineStr">
+        <is>
+          <t>Берёза</t>
+        </is>
+      </c>
+      <c r="X134" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB134" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC134" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE134" t="inlineStr">
+        <is>
+          <t>2026-10-19T04:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF134" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH134" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI134" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ134" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK134" t="inlineStr">
+        <is>
+          <t>2026-10-19T04:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>5542586163</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Брус и доска, документы ФГИС ЛК</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Собираем документы на брус и доску для тех, кто продаёт пиломатериал юрлицам.&lt;br&gt;&lt;br&gt;Когда покупатель крупный, у него свои требования: происхождение древесины, сопроводительные документы, чтобы всё сходилось в системе. Без этого сделку часто просто не проводят, даже если товар устраивает.&lt;br&gt;&lt;br&gt;Что делаем: заводим объём в ФГИС ЛК, оформляем основание договором купли-продажи, готовим ЭСД с QR кодом на отгрузки и полный комплект, который спокойно уходит в бухгалтерию покупателя.&lt;br&gt;&lt;br&gt;Работаем с пилорамами и перекупщиками по всей стране, удалённо.&lt;br&gt;&lt;br&gt;Брус, доска обрезная, пиломатериал хвоя, кругляк, Архангельская область.</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n04/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_08_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_08_3.jpg</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Архангельская обл., Вельск, ул. Дзержинского, 48</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P135" t="n">
+        <v>350</v>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V135" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W135" t="inlineStr">
+        <is>
+          <t>Сосна</t>
+        </is>
+      </c>
+      <c r="X135" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB135" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC135" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE135" t="inlineStr">
+        <is>
+          <t>2026-10-19T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF135" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH135" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI135" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ135" t="inlineStr">
+        <is>
+          <t>2026-09-19T11:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK135" t="inlineStr">
+        <is>
+          <t>2026-10-19T08:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>4323234383</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Осина дрова, документы на вывоз</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Документы на осину и дровяную древесину для тех, кто возит её на продажу.&lt;br&gt;&lt;br&gt;Многие считают, что дрова учитывать не надо. На деле это такая же древесина, и на рейс нужен электронный сопроводительный документ. Особенно если покупатель юрлицо и проводит покупку по бухгалтерии.&lt;br&gt;&lt;br&gt;Делаем полный круг: происхождение объёма через договор, внесение в ФГИС ЛК, ЭСД с QR кодом на каждую машину. Для постоянных перевозок считаем помесячно.&lt;br&gt;&lt;br&gt;От вас порода, объём, номер машины и маршрут. Остальное на нас.&lt;br&gt;&lt;br&gt;Осина дрова, баланс, берёза, горбыль, Брянская область.</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n14/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/batch/04/04_02.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/batch/04/04_03.jpg</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Брянская обл., Трубчевск, ул. Ленина, 60</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P136" t="n">
+        <v>250</v>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V136" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>Осина</t>
+        </is>
+      </c>
+      <c r="X136" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB136" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC136" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE136" t="inlineStr">
+        <is>
+          <t>2026-10-20T02:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF136" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH136" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI136" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ136" t="inlineStr">
+        <is>
+          <t>2026-09-20T05:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK136" t="inlineStr">
+        <is>
+          <t>2026-10-20T02:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>4637367814</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Доска и брусок, ЭСД на машину</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Оформляем сопроводительные документы на машины с пиломатериалом. Доска, брусок, обапол, тарная дощечка.&lt;br&gt;&lt;br&gt;Вопрос от пилорам звучит одинаково: нужен ли документ, если лес уже распилен. Нужен. Учёт никуда не исчезает после переработки, и на дороге это проверяют.&lt;br&gt;&lt;br&gt;Мы вносим объёмы в ФГИС ЛК, оформляем происхождение договором, готовим ЭСД с QR кодом на каждую отгрузку и собираем пакет, который спокойно принимает бухгалтерия покупателя.&lt;br&gt;&lt;br&gt;Если отгружаете регулярно, берём на сопровождение, так дешевле и быстрее.&lt;br&gt;&lt;br&gt;Доска обрезная, брусок, брус, пиломатериал хвоя, Брянская область.</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260813/n06/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_05_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_05_3.jpg</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Брянская обл., Жуковка, ул. Октябрьская, 3</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P137" t="n">
+        <v>350</v>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W137" t="inlineStr">
+        <is>
+          <t>Сосна</t>
+        </is>
+      </c>
+      <c r="X137" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB137" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC137" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE137" t="inlineStr">
+        <is>
+          <t>2026-10-20T04:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF137" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH137" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI137" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ137" t="inlineStr">
+        <is>
+          <t>2026-09-20T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK137" t="inlineStr">
+        <is>
+          <t>2026-10-20T04:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>1410610101</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Пиломатериал хвоя, документы ФГИС</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Ведём документы на хвойный пиломатериал: доска, брус, оцилиндрованное бревно, погонаж.&lt;br&gt;&lt;br&gt;Покупатель из другого региона почти всегда просит показать происхождение древесины. Без этого товар смотрят, но сделку не проводят, и хороший объём зависает на площадке.&lt;br&gt;&lt;br&gt;Закрываем это полностью. Оформляем договор купли-продажи как основание, заводим объёмы в систему учёта, выдаём сопроводительный документ с QR кодом на каждую отгрузку, готовим отчётность.&lt;br&gt;&lt;br&gt;Работаем с пилорамами и перекупщиками, удалённо, по всей стране.&lt;br&gt;&lt;br&gt;Пиломатериал хвоя, доска обрезная, брус, кругляк, Калужская область.</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_15_1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_13_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-21/fgis_2607_13_3.jpg</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Калужская обл., Людиново, ул. Ленина, 20</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P138" t="n">
+        <v>350</v>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W138" t="inlineStr">
+        <is>
+          <t>Сосна</t>
+        </is>
+      </c>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB138" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC138" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE138" t="inlineStr">
+        <is>
+          <t>2026-10-20T06:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF138" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH138" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI138" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ138" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK138" t="inlineStr">
+        <is>
+          <t>2026-10-20T06:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>6900416887</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Берёза кругляк, QR код на рейс</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Берёза с расчистки полей и обочин, документы делаем мы.&lt;br&gt;&lt;br&gt;Такой лес по закону учитывается так же, как из делянки. Владельцы участков узнают об этом обычно уже после того, как спилили, и упираются в то, что вывезти объём нельзя.&lt;br&gt;&lt;br&gt;Порядок работы: проводим происхождение через договор купли-продажи, вносим партию в ФГИС ЛК, ставим её вам на баланс. Дальше на каждую машину выписываем ЭСД с QR кодом, делаем это быстро, обычно за пятнадцать минут.&lt;br&gt;&lt;br&gt;Объём любой, от одной машины до постоянных отгрузок на комбинат.&lt;br&gt;&lt;br&gt;Берёза кругляк, дрова, баланс, фанкряж, Рязанская область.</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/batch/01/01_01.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_15_3.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_18_2.jpg</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Ремонт и строительство</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Рязанская обл., Касимов, ул. Советская, 14</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>ПВЗ</t>
+        </is>
+      </c>
+      <c r="P139" t="n">
+        <v>280</v>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>Стройматериалы</t>
+        </is>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>Товар приобретен на продажу</t>
+        </is>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>Пиломатериалы</t>
+        </is>
+      </c>
+      <c r="V139" t="inlineStr">
+        <is>
+          <t>Лес-кругляк</t>
+        </is>
+      </c>
+      <c r="W139" t="inlineStr">
+        <is>
+          <t>Берёза</t>
+        </is>
+      </c>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AB139" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="AC139" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="AE139" t="inlineStr">
+        <is>
+          <t>2026-10-20T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AF139" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AH139" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AI139" t="inlineStr">
+        <is>
+          <t>не опт</t>
+        </is>
+      </c>
+      <c r="AJ139" t="inlineStr">
+        <is>
+          <t>2026-09-20T11:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AK139" t="inlineStr">
+        <is>
+          <t>2026-10-20T08:00:00+03:00</t>
         </is>
       </c>
     </row>
@@ -26816,7 +29906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD22"/>
+  <dimension ref="A1:AD24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="21"/>
@@ -29582,6 +32672,266 @@
       <c r="AD22" t="inlineStr">
         <is>
           <t>2026-10-10T12:30:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>4740067166</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/wave_20260806/8194168577/1.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_07_2.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_07_3.jpg</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Предложение услуг</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>350</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ЭСД и QR код на перевозку леса</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Оформляем электронные сопроводительные документы на перевозку древесины.&lt;br&gt;&lt;br&gt;Это тот документ с QR кодом, который сейчас требуют на каждую машину с лесом. Делаем его на кругляк, на дрова, на пиломатериал, на любую породу.&lt;br&gt;&lt;br&gt;От вас данные: порода, объём, номер машины, откуда и куда. От нас готовый документ, обычно в течение пятнадцати минут. Если объёма в системе нет, сначала проводим происхождение через договор купли-продажи и ставим партию на баланс.&lt;br&gt;&lt;br&gt;Свой кабинет в ФГИС ЛК и электронную подпись заводить не нужно, всё делаем со своей стороны.&lt;br&gt;&lt;br&gt;Есть сопровождение помесячно для тех, кто отгружает постоянно.</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Республика Карелия, Медвежьегорск, ул. Кирова, 7</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Услуги посредников</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Консультации</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>4–7 лет</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>У себя</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>2026-10-16T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>2026-09-16T11:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>2026-10-16T08:00:00+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>8269348027</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>79824510018</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/fgis_doc_mo/01_01.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_18_3.jpg|https://raw.githubusercontent.com/Harmageddon14/avito-feeds/main/img/433120750/campaign_2026-07-29/fgis_0729_11_3.jpg</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Предложение услуг</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>350</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Закроем расхождения в ФГИС ЛК</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Разбираем расхождения в ФГИС ЛК. Это когда по системе у вас один объём, а по факту другой, и отгрузки из-за этого встают.&lt;br&gt;&lt;br&gt;Причины обычно простые: внесли не ту породу или сортимент, задвоили партию, списали меньше, чем увезли, приняли объём без основания. Дальше ошибка тянется, а на стороне покупателя она видна сразу.&lt;br&gt;&lt;br&gt;Мы поднимаем историю по вашему кабинету, находим, где разошлось, и приводим данные в порядок. Там, где нужно основание на объём, оформляем договор купли-продажи со своей стороны.&lt;br&gt;&lt;br&gt;После этого отгрузки идут нормально, а отчётность за период сдаётся без вопросов.&lt;br&gt;&lt;br&gt;Пишите, что происходит, посмотрим и скажем, сколько это займёт.</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Рязанская обл., Спас-Клепики, ул. Просвещения, 64</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Услуги посредников</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Консультации</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>4–7 лет</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>У себя</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>belpool.1@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>ФГИС ЛК объемы</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>2026-10-20T10:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>2026-09-20T13:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>2026-10-20T10:00:00+03:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fgislk: 6 объяв на 02.10, 3 на 03.10
</commit_message>
<xml_diff>
--- a/fgislk.xlsx
+++ b/fgislk.xlsx
@@ -10252,17 +10252,17 @@
       </c>
       <c r="AC43" t="inlineStr">
         <is>
-          <t>2026-11-02T08:00:00+03:00</t>
+          <t>2026-11-02T02:00:00+03:00</t>
         </is>
       </c>
       <c r="AD43" t="inlineStr">
         <is>
-          <t>2026-10-03T11:00:00+03:00</t>
+          <t>2026-10-03T05:00:00+03:00</t>
         </is>
       </c>
       <c r="AE43" t="inlineStr">
         <is>
-          <t>2026-11-02T08:00:00+03:00</t>
+          <t>2026-11-02T02:00:00+03:00</t>
         </is>
       </c>
     </row>
@@ -10382,17 +10382,17 @@
       </c>
       <c r="AC44" t="inlineStr">
         <is>
-          <t>2026-11-02T12:00:00+03:00</t>
+          <t>2026-11-02T06:00:00+03:00</t>
         </is>
       </c>
       <c r="AD44" t="inlineStr">
         <is>
-          <t>2026-10-03T15:00:00+03:00</t>
+          <t>2026-10-03T09:00:00+03:00</t>
         </is>
       </c>
       <c r="AE44" t="inlineStr">
         <is>
-          <t>2026-11-02T12:00:00+03:00</t>
+          <t>2026-11-02T06:00:00+03:00</t>
         </is>
       </c>
     </row>
@@ -30719,7 +30719,7 @@
       </c>
       <c r="AE144" t="inlineStr">
         <is>
-          <t>2026-11-02T04:00:00+03:00</t>
+          <t>2026-11-01T13:30:00+03:00</t>
         </is>
       </c>
       <c r="AF144" t="inlineStr">
@@ -30739,12 +30739,12 @@
       </c>
       <c r="AJ144" t="inlineStr">
         <is>
-          <t>2026-10-03T07:00:00+03:00</t>
+          <t>2026-10-02T16:30:00+03:00</t>
         </is>
       </c>
       <c r="AK144" t="inlineStr">
         <is>
-          <t>2026-11-02T04:00:00+03:00</t>
+          <t>2026-11-01T13:30:00+03:00</t>
         </is>
       </c>
     </row>
@@ -30854,7 +30854,7 @@
       </c>
       <c r="AE145" t="inlineStr">
         <is>
-          <t>2026-11-02T10:00:00+03:00</t>
+          <t>2026-11-02T04:00:00+03:00</t>
         </is>
       </c>
       <c r="AF145" t="inlineStr">
@@ -30874,12 +30874,12 @@
       </c>
       <c r="AJ145" t="inlineStr">
         <is>
-          <t>2026-10-03T13:00:00+03:00</t>
+          <t>2026-10-03T07:00:00+03:00</t>
         </is>
       </c>
       <c r="AK145" t="inlineStr">
         <is>
-          <t>2026-11-02T10:00:00+03:00</t>
+          <t>2026-11-02T04:00:00+03:00</t>
         </is>
       </c>
     </row>
@@ -36071,17 +36071,17 @@
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>2026-11-02T02:00:00+03:00</t>
+          <t>2026-11-01T11:30:00+03:00</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>2026-10-03T05:00:00+03:00</t>
+          <t>2026-10-02T14:30:00+03:00</t>
         </is>
       </c>
       <c r="AD30" t="inlineStr">
         <is>
-          <t>2026-11-02T02:00:00+03:00</t>
+          <t>2026-11-01T11:30:00+03:00</t>
         </is>
       </c>
     </row>
@@ -36201,17 +36201,17 @@
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>2026-11-02T06:00:00+03:00</t>
+          <t>2026-11-01T15:00:00+03:00</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>2026-10-03T09:00:00+03:00</t>
+          <t>2026-10-02T18:00:00+03:00</t>
         </is>
       </c>
       <c r="AD31" t="inlineStr">
         <is>
-          <t>2026-11-02T06:00:00+03:00</t>
+          <t>2026-11-01T15:00:00+03:00</t>
         </is>
       </c>
     </row>

</xml_diff>